<commit_message>
Data Model updates based ont the new requirement.
</commit_message>
<xml_diff>
--- a/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
+++ b/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\Requirement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBBFBD9A-11F1-415F-A591-C302C1404054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973F0398-F95F-496D-B8BD-C515317055B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3649FE5F-4067-43E3-9705-A3C81FD1AFF4}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="19">
   <si>
     <t>Description</t>
   </si>
@@ -76,6 +76,12 @@
   </si>
   <si>
     <t>High</t>
+  </si>
+  <si>
+    <t>Provide facility for Upgrade of Membership  from Silver to Gold - Platninum, Caluate the new cost on pro rata basis but reset the subscription period basedon that tier period/duration</t>
+  </si>
+  <si>
+    <t>Add an approval workflow for the Org admin changes specially Membership/Offers by the owner or specific designated entity.</t>
   </si>
 </sst>
 </file>
@@ -509,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7621361-7740-4C28-A3A1-E7CF2DAB5704}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -636,6 +642,40 @@
         <v>14</v>
       </c>
     </row>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>